<commit_message>
Update report: 동면 20260316_20260317
</commit_message>
<xml_diff>
--- a/shucle_report/동면/20260316_20260317/report_동면_20260316_20260317.xlsx
+++ b/shucle_report/동면/20260316_20260317/report_동면_20260316_20260317.xlsx
@@ -514,7 +514,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>분석기간: 2026.03.16 ~ 03.17 | 비교기간: 2026.03.12 ~ 03.13 | 생성: 2026-03-18 16:53 | 차트: 98개</t>
+          <t>분석기간: 2026.03.16 ~ 03.17 | 비교기간: 2026.03.12 ~ 03.13 | 생성: 2026-03-18 16:55 | 차트: 98개</t>
         </is>
       </c>
     </row>
@@ -1104,7 +1104,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G50"/>
+  <dimension ref="A1:G52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1825,32 +1825,32 @@
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>동승 인원 분포(일평균)</t>
+          <t>대당 탑승객 수(평일)</t>
         </is>
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>9.50</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>7.00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E28" s="7" t="inlineStr">
         <is>
-          <t>-2.50</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F28" s="7" t="inlineStr">
         <is>
-          <t>-26.3%</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G28" s="6" t="inlineStr">
         <is>
-          <t>동승 비율 변화에 따른 대당 탑승 변화</t>
+          <t>평일 차량당 탑승객 변화</t>
         </is>
       </c>
     </row>
@@ -1862,32 +1862,32 @@
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>실시간 호출 건수(일평균)</t>
+          <t>대당 탑승객 수(주말)</t>
         </is>
       </c>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>10.0</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>4.00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E29" s="7" t="inlineStr">
         <is>
-          <t>-6.00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F29" s="7" t="inlineStr">
         <is>
-          <t>-60.0%</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G29" s="6" t="inlineStr">
         <is>
-          <t>수요 변동에 따른 대당 배분 변화</t>
+          <t>주말 차량당 탑승객 변화</t>
         </is>
       </c>
     </row>
@@ -1899,150 +1899,150 @@
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
+          <t>동승 인원 분포(일평균)</t>
+        </is>
+      </c>
+      <c r="C30" s="7" t="inlineStr">
+        <is>
+          <t>9.50</t>
+        </is>
+      </c>
+      <c r="D30" s="7" t="inlineStr">
+        <is>
+          <t>7.00</t>
+        </is>
+      </c>
+      <c r="E30" s="7" t="inlineStr">
+        <is>
+          <t>-2.50</t>
+        </is>
+      </c>
+      <c r="F30" s="7" t="inlineStr">
+        <is>
+          <t>-26.3%</t>
+        </is>
+      </c>
+      <c r="G30" s="6" t="inlineStr">
+        <is>
+          <t>동승 비율 변화에 따른 대당 탑승 변화</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
+          <t>대당 탑승객 수</t>
+        </is>
+      </c>
+      <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t>실시간 호출 건수(일평균)</t>
+        </is>
+      </c>
+      <c r="C31" s="7" t="inlineStr">
+        <is>
+          <t>10.0</t>
+        </is>
+      </c>
+      <c r="D31" s="7" t="inlineStr">
+        <is>
+          <t>4.00</t>
+        </is>
+      </c>
+      <c r="E31" s="7" t="inlineStr">
+        <is>
+          <t>-6.00</t>
+        </is>
+      </c>
+      <c r="F31" s="7" t="inlineStr">
+        <is>
+          <t>-60.0%</t>
+        </is>
+      </c>
+      <c r="G31" s="6" t="inlineStr">
+        <is>
+          <t>수요 변동에 따른 대당 배분 변화</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t>대당 탑승객 수</t>
+        </is>
+      </c>
+      <c r="B32" s="6" t="inlineStr">
+        <is>
           <t>운행차량 대수</t>
         </is>
       </c>
-      <c r="C30" s="7" t="inlineStr">
+      <c r="C32" s="7" t="inlineStr">
         <is>
           <t>1.00</t>
         </is>
       </c>
-      <c r="D30" s="7" t="inlineStr">
+      <c r="D32" s="7" t="inlineStr">
         <is>
           <t>1.00</t>
         </is>
       </c>
-      <c r="E30" s="7" t="inlineStr">
+      <c r="E32" s="7" t="inlineStr">
         <is>
           <t>+0.00</t>
         </is>
       </c>
-      <c r="F30" s="7" t="inlineStr">
+      <c r="F32" s="7" t="inlineStr">
         <is>
           <t>+0.0%</t>
         </is>
       </c>
-      <c r="G30" s="6" t="inlineStr">
+      <c r="G32" s="6" t="inlineStr">
         <is>
           <t>차량 수 변동에 따른 대당 배분 변화</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="10" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="10" t="inlineStr">
         <is>
           <t>▲ 평균 우회비율 (+13.7%)</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="4" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
         <is>
           <t>구분</t>
         </is>
       </c>
-      <c r="B33" s="4" t="inlineStr">
+      <c r="B35" s="4" t="inlineStr">
         <is>
           <t>세부지표</t>
         </is>
       </c>
-      <c r="C33" s="4" t="inlineStr">
+      <c r="C35" s="4" t="inlineStr">
         <is>
           <t>비교기간</t>
         </is>
       </c>
-      <c r="D33" s="4" t="inlineStr">
+      <c r="D35" s="4" t="inlineStr">
         <is>
           <t>분석기간</t>
         </is>
       </c>
-      <c r="E33" s="4" t="inlineStr">
+      <c r="E35" s="4" t="inlineStr">
         <is>
           <t>변동값</t>
         </is>
       </c>
-      <c r="F33" s="4" t="inlineStr">
+      <c r="F35" s="4" t="inlineStr">
         <is>
           <t>변동률</t>
         </is>
       </c>
-      <c r="G33" s="4" t="inlineStr">
+      <c r="G35" s="4" t="inlineStr">
         <is>
           <t>포인트</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="6" t="inlineStr">
-        <is>
-          <t>평균 우회비율</t>
-        </is>
-      </c>
-      <c r="B34" s="6" t="inlineStr">
-        <is>
-          <t>상위 10% 우회비율</t>
-        </is>
-      </c>
-      <c r="C34" s="7" t="inlineStr">
-        <is>
-          <t>1.45</t>
-        </is>
-      </c>
-      <c r="D34" s="7" t="inlineStr">
-        <is>
-          <t>1.39</t>
-        </is>
-      </c>
-      <c r="E34" s="7" t="inlineStr">
-        <is>
-          <t>-0.07</t>
-        </is>
-      </c>
-      <c r="F34" s="7" t="inlineStr">
-        <is>
-          <t>-4.5%</t>
-        </is>
-      </c>
-      <c r="G34" s="6" t="inlineStr">
-        <is>
-          <t>극단적 우회 경로 발생</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="6" t="inlineStr">
-        <is>
-          <t>평균 우회비율</t>
-        </is>
-      </c>
-      <c r="B35" s="6" t="inlineStr">
-        <is>
-          <t>평균 이동시간</t>
-        </is>
-      </c>
-      <c r="C35" s="7" t="inlineStr">
-        <is>
-          <t>10.3</t>
-        </is>
-      </c>
-      <c r="D35" s="7" t="inlineStr">
-        <is>
-          <t>10.4</t>
-        </is>
-      </c>
-      <c r="E35" s="7" t="inlineStr">
-        <is>
-          <t>+0.17</t>
-        </is>
-      </c>
-      <c r="F35" s="7" t="inlineStr">
-        <is>
-          <t>+1.7%</t>
-        </is>
-      </c>
-      <c r="G35" s="6" t="inlineStr">
-        <is>
-          <t>우회 경로 증가가 이동시간 상승 유발</t>
         </is>
       </c>
     </row>
@@ -2054,150 +2054,150 @@
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
+          <t>상위 10% 우회비율</t>
+        </is>
+      </c>
+      <c r="C36" s="7" t="inlineStr">
+        <is>
+          <t>1.45</t>
+        </is>
+      </c>
+      <c r="D36" s="7" t="inlineStr">
+        <is>
+          <t>1.39</t>
+        </is>
+      </c>
+      <c r="E36" s="7" t="inlineStr">
+        <is>
+          <t>-0.07</t>
+        </is>
+      </c>
+      <c r="F36" s="7" t="inlineStr">
+        <is>
+          <t>-4.5%</t>
+        </is>
+      </c>
+      <c r="G36" s="6" t="inlineStr">
+        <is>
+          <t>극단적 우회 경로 발생</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="6" t="inlineStr">
+        <is>
+          <t>평균 우회비율</t>
+        </is>
+      </c>
+      <c r="B37" s="6" t="inlineStr">
+        <is>
+          <t>평균 이동시간</t>
+        </is>
+      </c>
+      <c r="C37" s="7" t="inlineStr">
+        <is>
+          <t>10.3</t>
+        </is>
+      </c>
+      <c r="D37" s="7" t="inlineStr">
+        <is>
+          <t>10.4</t>
+        </is>
+      </c>
+      <c r="E37" s="7" t="inlineStr">
+        <is>
+          <t>+0.17</t>
+        </is>
+      </c>
+      <c r="F37" s="7" t="inlineStr">
+        <is>
+          <t>+1.7%</t>
+        </is>
+      </c>
+      <c r="G37" s="6" t="inlineStr">
+        <is>
+          <t>우회 경로 증가가 이동시간 상승 유발</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="6" t="inlineStr">
+        <is>
+          <t>평균 우회비율</t>
+        </is>
+      </c>
+      <c r="B38" s="6" t="inlineStr">
+        <is>
           <t>동승 인원 분포(일평균)</t>
         </is>
       </c>
-      <c r="C36" s="7" t="inlineStr">
+      <c r="C38" s="7" t="inlineStr">
         <is>
           <t>9.50</t>
         </is>
       </c>
-      <c r="D36" s="7" t="inlineStr">
+      <c r="D38" s="7" t="inlineStr">
         <is>
           <t>7.00</t>
         </is>
       </c>
-      <c r="E36" s="7" t="inlineStr">
+      <c r="E38" s="7" t="inlineStr">
         <is>
           <t>-2.50</t>
         </is>
       </c>
-      <c r="F36" s="7" t="inlineStr">
+      <c r="F38" s="7" t="inlineStr">
         <is>
           <t>-26.3%</t>
         </is>
       </c>
-      <c r="G36" s="6" t="inlineStr">
+      <c r="G38" s="6" t="inlineStr">
         <is>
           <t>동승 증가로 경유지 추가</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="10" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="10" t="inlineStr">
         <is>
           <t>▼ 평균 대당 운행거리 (-28.5%)</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="4" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
         <is>
           <t>구분</t>
         </is>
       </c>
-      <c r="B39" s="4" t="inlineStr">
+      <c r="B41" s="4" t="inlineStr">
         <is>
           <t>세부지표</t>
         </is>
       </c>
-      <c r="C39" s="4" t="inlineStr">
+      <c r="C41" s="4" t="inlineStr">
         <is>
           <t>비교기간</t>
         </is>
       </c>
-      <c r="D39" s="4" t="inlineStr">
+      <c r="D41" s="4" t="inlineStr">
         <is>
           <t>분석기간</t>
         </is>
       </c>
-      <c r="E39" s="4" t="inlineStr">
+      <c r="E41" s="4" t="inlineStr">
         <is>
           <t>변동값</t>
         </is>
       </c>
-      <c r="F39" s="4" t="inlineStr">
+      <c r="F41" s="4" t="inlineStr">
         <is>
           <t>변동률</t>
         </is>
       </c>
-      <c r="G39" s="4" t="inlineStr">
+      <c r="G41" s="4" t="inlineStr">
         <is>
           <t>포인트</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="6" t="inlineStr">
-        <is>
-          <t>평균 대당 운행거리</t>
-        </is>
-      </c>
-      <c r="B40" s="6" t="inlineStr">
-        <is>
-          <t>일간 평균 대당 운행거리</t>
-        </is>
-      </c>
-      <c r="C40" s="7" t="inlineStr">
-        <is>
-          <t>89.5</t>
-        </is>
-      </c>
-      <c r="D40" s="7" t="inlineStr">
-        <is>
-          <t>64.0</t>
-        </is>
-      </c>
-      <c r="E40" s="7" t="inlineStr">
-        <is>
-          <t>-25.5</t>
-        </is>
-      </c>
-      <c r="F40" s="7" t="inlineStr">
-        <is>
-          <t>-28.5%</t>
-        </is>
-      </c>
-      <c r="G40" s="6" t="inlineStr">
-        <is>
-          <t>일별 운행거리 편차</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="6" t="inlineStr">
-        <is>
-          <t>평균 대당 운행거리</t>
-        </is>
-      </c>
-      <c r="B41" s="6" t="inlineStr">
-        <is>
-          <t>실시간 호출 건수(일평균)</t>
-        </is>
-      </c>
-      <c r="C41" s="7" t="inlineStr">
-        <is>
-          <t>10.0</t>
-        </is>
-      </c>
-      <c r="D41" s="7" t="inlineStr">
-        <is>
-          <t>4.00</t>
-        </is>
-      </c>
-      <c r="E41" s="7" t="inlineStr">
-        <is>
-          <t>-6.00</t>
-        </is>
-      </c>
-      <c r="F41" s="7" t="inlineStr">
-        <is>
-          <t>-60.0%</t>
-        </is>
-      </c>
-      <c r="G41" s="6" t="inlineStr">
-        <is>
-          <t>수요 변동에 따른 운행거리 변화</t>
         </is>
       </c>
     </row>
@@ -2209,150 +2209,150 @@
       </c>
       <c r="B42" s="6" t="inlineStr">
         <is>
+          <t>일간 평균 대당 운행거리</t>
+        </is>
+      </c>
+      <c r="C42" s="7" t="inlineStr">
+        <is>
+          <t>89.5</t>
+        </is>
+      </c>
+      <c r="D42" s="7" t="inlineStr">
+        <is>
+          <t>64.0</t>
+        </is>
+      </c>
+      <c r="E42" s="7" t="inlineStr">
+        <is>
+          <t>-25.5</t>
+        </is>
+      </c>
+      <c r="F42" s="7" t="inlineStr">
+        <is>
+          <t>-28.5%</t>
+        </is>
+      </c>
+      <c r="G42" s="6" t="inlineStr">
+        <is>
+          <t>일별 운행거리 편차</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="6" t="inlineStr">
+        <is>
+          <t>평균 대당 운행거리</t>
+        </is>
+      </c>
+      <c r="B43" s="6" t="inlineStr">
+        <is>
+          <t>실시간 호출 건수(일평균)</t>
+        </is>
+      </c>
+      <c r="C43" s="7" t="inlineStr">
+        <is>
+          <t>10.0</t>
+        </is>
+      </c>
+      <c r="D43" s="7" t="inlineStr">
+        <is>
+          <t>4.00</t>
+        </is>
+      </c>
+      <c r="E43" s="7" t="inlineStr">
+        <is>
+          <t>-6.00</t>
+        </is>
+      </c>
+      <c r="F43" s="7" t="inlineStr">
+        <is>
+          <t>-60.0%</t>
+        </is>
+      </c>
+      <c r="G43" s="6" t="inlineStr">
+        <is>
+          <t>수요 변동에 따른 운행거리 변화</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="6" t="inlineStr">
+        <is>
+          <t>평균 대당 운행거리</t>
+        </is>
+      </c>
+      <c r="B44" s="6" t="inlineStr">
+        <is>
           <t>운행차량 대수</t>
         </is>
       </c>
-      <c r="C42" s="7" t="inlineStr">
+      <c r="C44" s="7" t="inlineStr">
         <is>
           <t>1.00</t>
         </is>
       </c>
-      <c r="D42" s="7" t="inlineStr">
+      <c r="D44" s="7" t="inlineStr">
         <is>
           <t>1.00</t>
         </is>
       </c>
-      <c r="E42" s="7" t="inlineStr">
+      <c r="E44" s="7" t="inlineStr">
         <is>
           <t>+0.00</t>
         </is>
       </c>
-      <c r="F42" s="7" t="inlineStr">
+      <c r="F44" s="7" t="inlineStr">
         <is>
           <t>+0.0%</t>
         </is>
       </c>
-      <c r="G42" s="6" t="inlineStr">
+      <c r="G44" s="6" t="inlineStr">
         <is>
           <t>차량 수 변동에 따른 대당 거리 변화</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="10" t="inlineStr">
+    <row r="46">
+      <c r="A46" s="10" t="inlineStr">
         <is>
           <t>▼ DAU (일간 활성 회원) (-12.5%)</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="4" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
         <is>
           <t>구분</t>
         </is>
       </c>
-      <c r="B45" s="4" t="inlineStr">
+      <c r="B47" s="4" t="inlineStr">
         <is>
           <t>세부지표</t>
         </is>
       </c>
-      <c r="C45" s="4" t="inlineStr">
+      <c r="C47" s="4" t="inlineStr">
         <is>
           <t>비교기간</t>
         </is>
       </c>
-      <c r="D45" s="4" t="inlineStr">
+      <c r="D47" s="4" t="inlineStr">
         <is>
           <t>분석기간</t>
         </is>
       </c>
-      <c r="E45" s="4" t="inlineStr">
+      <c r="E47" s="4" t="inlineStr">
         <is>
           <t>변동값</t>
         </is>
       </c>
-      <c r="F45" s="4" t="inlineStr">
+      <c r="F47" s="4" t="inlineStr">
         <is>
           <t>변동률</t>
         </is>
       </c>
-      <c r="G45" s="4" t="inlineStr">
+      <c r="G47" s="4" t="inlineStr">
         <is>
           <t>포인트</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="6" t="inlineStr">
-        <is>
-          <t>DAU (일간 활성 회원)</t>
-        </is>
-      </c>
-      <c r="B46" s="6" t="inlineStr">
-        <is>
-          <t>WAU (주간 활성 회원)</t>
-        </is>
-      </c>
-      <c r="C46" s="7" t="inlineStr">
-        <is>
-          <t>7.00</t>
-        </is>
-      </c>
-      <c r="D46" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E46" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F46" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G46" s="6" t="inlineStr">
-        <is>
-          <t>주간 활성도 추이 연동</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="6" t="inlineStr">
-        <is>
-          <t>DAU (일간 활성 회원)</t>
-        </is>
-      </c>
-      <c r="B47" s="6" t="inlineStr">
-        <is>
-          <t>신규 지역 회원(일평균)</t>
-        </is>
-      </c>
-      <c r="C47" s="7" t="inlineStr">
-        <is>
-          <t>3.00</t>
-        </is>
-      </c>
-      <c r="D47" s="7" t="inlineStr">
-        <is>
-          <t>3.00</t>
-        </is>
-      </c>
-      <c r="E47" s="7" t="inlineStr">
-        <is>
-          <t>+0.00</t>
-        </is>
-      </c>
-      <c r="F47" s="7" t="inlineStr">
-        <is>
-          <t>+0.0%</t>
-        </is>
-      </c>
-      <c r="G47" s="6" t="inlineStr">
-        <is>
-          <t>신규 유입 증감 영향</t>
         </is>
       </c>
     </row>
@@ -2364,32 +2364,32 @@
       </c>
       <c r="B48" s="6" t="inlineStr">
         <is>
-          <t>활성 회원 평균연령</t>
+          <t>WAU (주간 활성 회원)</t>
         </is>
       </c>
       <c r="C48" s="7" t="inlineStr">
         <is>
-          <t>65.0</t>
+          <t>7.00</t>
         </is>
       </c>
       <c r="D48" s="7" t="inlineStr">
         <is>
-          <t>75.0</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E48" s="7" t="inlineStr">
         <is>
-          <t>+10.0</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F48" s="7" t="inlineStr">
         <is>
-          <t>+15.4%</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G48" s="6" t="inlineStr">
         <is>
-          <t>이용자 평균 연령 변화</t>
+          <t>주간 활성도 추이 연동</t>
         </is>
       </c>
     </row>
@@ -2401,32 +2401,32 @@
       </c>
       <c r="B49" s="6" t="inlineStr">
         <is>
-          <t>가호출 성공률</t>
+          <t>신규 지역 회원(일평균)</t>
         </is>
       </c>
       <c r="C49" s="7" t="inlineStr">
         <is>
-          <t>0.39</t>
+          <t>3.00</t>
         </is>
       </c>
       <c r="D49" s="7" t="inlineStr">
         <is>
-          <t>0.88</t>
+          <t>3.00</t>
         </is>
       </c>
       <c r="E49" s="7" t="inlineStr">
         <is>
-          <t>+0.49</t>
+          <t>+0.00</t>
         </is>
       </c>
       <c r="F49" s="7" t="inlineStr">
         <is>
-          <t>+127.0%</t>
+          <t>+0.0%</t>
         </is>
       </c>
       <c r="G49" s="6" t="inlineStr">
         <is>
-          <t>서비스 품질 불만에 따른 이탈</t>
+          <t>신규 유입 증감 영향</t>
         </is>
       </c>
     </row>
@@ -2438,30 +2438,104 @@
       </c>
       <c r="B50" s="6" t="inlineStr">
         <is>
+          <t>활성 회원 평균연령</t>
+        </is>
+      </c>
+      <c r="C50" s="7" t="inlineStr">
+        <is>
+          <t>65.0</t>
+        </is>
+      </c>
+      <c r="D50" s="7" t="inlineStr">
+        <is>
+          <t>75.0</t>
+        </is>
+      </c>
+      <c r="E50" s="7" t="inlineStr">
+        <is>
+          <t>+10.0</t>
+        </is>
+      </c>
+      <c r="F50" s="7" t="inlineStr">
+        <is>
+          <t>+15.4%</t>
+        </is>
+      </c>
+      <c r="G50" s="6" t="inlineStr">
+        <is>
+          <t>이용자 평균 연령 변화</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="6" t="inlineStr">
+        <is>
+          <t>DAU (일간 활성 회원)</t>
+        </is>
+      </c>
+      <c r="B51" s="6" t="inlineStr">
+        <is>
+          <t>가호출 성공률</t>
+        </is>
+      </c>
+      <c r="C51" s="7" t="inlineStr">
+        <is>
+          <t>0.39</t>
+        </is>
+      </c>
+      <c r="D51" s="7" t="inlineStr">
+        <is>
+          <t>0.88</t>
+        </is>
+      </c>
+      <c r="E51" s="7" t="inlineStr">
+        <is>
+          <t>+0.49</t>
+        </is>
+      </c>
+      <c r="F51" s="7" t="inlineStr">
+        <is>
+          <t>+127.0%</t>
+        </is>
+      </c>
+      <c r="G51" s="6" t="inlineStr">
+        <is>
+          <t>서비스 품질 불만에 따른 이탈</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="6" t="inlineStr">
+        <is>
+          <t>DAU (일간 활성 회원)</t>
+        </is>
+      </c>
+      <c r="B52" s="6" t="inlineStr">
+        <is>
           <t>평균 대기시간</t>
         </is>
       </c>
-      <c r="C50" s="7" t="inlineStr">
+      <c r="C52" s="7" t="inlineStr">
         <is>
           <t>2.76</t>
         </is>
       </c>
-      <c r="D50" s="7" t="inlineStr">
+      <c r="D52" s="7" t="inlineStr">
         <is>
           <t>2.97</t>
         </is>
       </c>
-      <c r="E50" s="7" t="inlineStr">
+      <c r="E52" s="7" t="inlineStr">
         <is>
           <t>+0.22</t>
         </is>
       </c>
-      <c r="F50" s="7" t="inlineStr">
+      <c r="F52" s="7" t="inlineStr">
         <is>
           <t>+7.9%</t>
         </is>
       </c>
-      <c r="G50" s="6" t="inlineStr">
+      <c r="G52" s="6" t="inlineStr">
         <is>
           <t>대기시간 증가에 따른 이탈</t>
         </is>
@@ -2469,14 +2543,14 @@
     </row>
   </sheetData>
   <mergeCells count="8">
-    <mergeCell ref="A32:G32"/>
     <mergeCell ref="A13:G13"/>
-    <mergeCell ref="A44:G44"/>
     <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A40:G40"/>
     <mergeCell ref="A3:G3"/>
+    <mergeCell ref="A34:G34"/>
     <mergeCell ref="A26:G26"/>
-    <mergeCell ref="A38:G38"/>
     <mergeCell ref="A19:G19"/>
+    <mergeCell ref="A46:G46"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2488,7 +2562,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G43"/>
+  <dimension ref="A1:G47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2559,32 +2633,32 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>상위 10% 대기시간</t>
+          <t>평균 대기시간(평일)</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>7.70</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>10.1</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>+2.40</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>+31.2%</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G5" s="6" t="inlineStr">
         <is>
-          <t>극단적 장시간 대기 사례 발생</t>
+          <t>평일 대기시간 변화</t>
         </is>
       </c>
     </row>
@@ -2596,22 +2670,22 @@
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>장시간 대기(30분+) 비율</t>
+          <t>평균 대기시간(주말)</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>+0.0%p</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F6" s="7" t="inlineStr">
@@ -2621,7 +2695,7 @@
       </c>
       <c r="G6" s="6" t="inlineStr">
         <is>
-          <t>30분 이상 장시간 대기 비중</t>
+          <t>주말 대기시간 변화</t>
         </is>
       </c>
     </row>
@@ -2633,32 +2707,32 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>운행차량 대수</t>
+          <t>상위 10% 대기시간</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>1.00</t>
+          <t>7.70</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>1.00</t>
+          <t>10.1</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>+0.00</t>
+          <t>+2.40</t>
         </is>
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>+0.0%</t>
+          <t>+31.2%</t>
         </is>
       </c>
       <c r="G7" s="6" t="inlineStr">
         <is>
-          <t>차량 공급 부족에 따른 대기 증가</t>
+          <t>극단적 장시간 대기 사례 발생</t>
         </is>
       </c>
     </row>
@@ -2670,150 +2744,150 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
+          <t>장시간 대기(30분+) 비율</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>+0.0%p</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>30분 이상 장시간 대기 비중</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>평균 대기시간</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>운행차량 대수</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>1.00</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>1.00</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>+0.00</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>차량 공급 부족에 따른 대기 증가</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>평균 대기시간</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
           <t>실시간 호출 건수(일평균)</t>
         </is>
       </c>
-      <c r="C8" s="7" t="inlineStr">
+      <c r="C10" s="7" t="inlineStr">
         <is>
           <t>10.0</t>
         </is>
       </c>
-      <c r="D8" s="7" t="inlineStr">
+      <c r="D10" s="7" t="inlineStr">
         <is>
           <t>4.00</t>
         </is>
       </c>
-      <c r="E8" s="7" t="inlineStr">
+      <c r="E10" s="7" t="inlineStr">
         <is>
           <t>-6.00</t>
         </is>
       </c>
-      <c r="F8" s="7" t="inlineStr">
+      <c r="F10" s="7" t="inlineStr">
         <is>
           <t>-60.0%</t>
         </is>
       </c>
-      <c r="G8" s="6" t="inlineStr">
+      <c r="G10" s="6" t="inlineStr">
         <is>
           <t>수요 대비 공급 불균형</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="10" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="10" t="inlineStr">
         <is>
           <t>▲ 평균 이동시간 (+1.7%)</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>구분</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B13" s="4" t="inlineStr">
         <is>
           <t>세부지표</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C13" s="4" t="inlineStr">
         <is>
           <t>비교기간</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
+      <c r="D13" s="4" t="inlineStr">
         <is>
           <t>분석기간</t>
         </is>
       </c>
-      <c r="E11" s="4" t="inlineStr">
+      <c r="E13" s="4" t="inlineStr">
         <is>
           <t>변동값</t>
         </is>
       </c>
-      <c r="F11" s="4" t="inlineStr">
+      <c r="F13" s="4" t="inlineStr">
         <is>
           <t>변동률</t>
         </is>
       </c>
-      <c r="G11" s="4" t="inlineStr">
+      <c r="G13" s="4" t="inlineStr">
         <is>
           <t>포인트</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t>평균 이동시간</t>
-        </is>
-      </c>
-      <c r="B12" s="6" t="inlineStr">
-        <is>
-          <t>피크 시간대(15~17시) 이동시간</t>
-        </is>
-      </c>
-      <c r="C12" s="7" t="inlineStr">
-        <is>
-          <t>11.5</t>
-        </is>
-      </c>
-      <c r="D12" s="7" t="inlineStr">
-        <is>
-          <t>9.30</t>
-        </is>
-      </c>
-      <c r="E12" s="7" t="inlineStr">
-        <is>
-          <t>-2.17</t>
-        </is>
-      </c>
-      <c r="F12" s="7" t="inlineStr">
-        <is>
-          <t>-19.0%</t>
-        </is>
-      </c>
-      <c r="G12" s="6" t="inlineStr">
-        <is>
-          <t>피크 시간대 이동시간 변화</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>평균 이동시간</t>
-        </is>
-      </c>
-      <c r="B13" s="6" t="inlineStr">
-        <is>
-          <t>비피크 시간대(8~10시) 이동시간</t>
-        </is>
-      </c>
-      <c r="C13" s="7" t="inlineStr">
-        <is>
-          <t>9.80</t>
-        </is>
-      </c>
-      <c r="D13" s="7" t="inlineStr">
-        <is>
-          <t>19.0</t>
-        </is>
-      </c>
-      <c r="E13" s="7" t="inlineStr">
-        <is>
-          <t>+9.20</t>
-        </is>
-      </c>
-      <c r="F13" s="7" t="inlineStr">
-        <is>
-          <t>+93.9%</t>
-        </is>
-      </c>
-      <c r="G13" s="6" t="inlineStr">
-        <is>
-          <t>비피크 시간대 이동시간 변화</t>
         </is>
       </c>
     </row>
@@ -2825,150 +2899,150 @@
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
+          <t>피크 시간대(15~17시) 이동시간</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>11.5</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>9.30</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>-2.17</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>-19.0%</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>피크 시간대 이동시간 변화</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>평균 이동시간</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>비피크 시간대(8~10시) 이동시간</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>9.80</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>19.0</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>+9.20</t>
+        </is>
+      </c>
+      <c r="F15" s="7" t="inlineStr">
+        <is>
+          <t>+93.9%</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>비피크 시간대 이동시간 변화</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>평균 이동시간</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
           <t>평균 우회비율</t>
         </is>
       </c>
-      <c r="C14" s="7" t="inlineStr">
+      <c r="C16" s="7" t="inlineStr">
         <is>
           <t>0.94</t>
         </is>
       </c>
-      <c r="D14" s="7" t="inlineStr">
+      <c r="D16" s="7" t="inlineStr">
         <is>
           <t>1.07</t>
         </is>
       </c>
-      <c r="E14" s="7" t="inlineStr">
+      <c r="E16" s="7" t="inlineStr">
         <is>
           <t>+0.13</t>
         </is>
       </c>
-      <c r="F14" s="7" t="inlineStr">
+      <c r="F16" s="7" t="inlineStr">
         <is>
           <t>+13.7%</t>
         </is>
       </c>
-      <c r="G14" s="6" t="inlineStr">
+      <c r="G16" s="6" t="inlineStr">
         <is>
           <t>경로 우회에 따른 이동시간 증가</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="10" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="10" t="inlineStr">
         <is>
           <t>─ 운행차량 대수 (+0.0%)</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>구분</t>
         </is>
       </c>
-      <c r="B17" s="4" t="inlineStr">
+      <c r="B19" s="4" t="inlineStr">
         <is>
           <t>세부지표</t>
         </is>
       </c>
-      <c r="C17" s="4" t="inlineStr">
+      <c r="C19" s="4" t="inlineStr">
         <is>
           <t>비교기간</t>
         </is>
       </c>
-      <c r="D17" s="4" t="inlineStr">
+      <c r="D19" s="4" t="inlineStr">
         <is>
           <t>분석기간</t>
         </is>
       </c>
-      <c r="E17" s="4" t="inlineStr">
+      <c r="E19" s="4" t="inlineStr">
         <is>
           <t>변동값</t>
         </is>
       </c>
-      <c r="F17" s="4" t="inlineStr">
+      <c r="F19" s="4" t="inlineStr">
         <is>
           <t>변동률</t>
         </is>
       </c>
-      <c r="G17" s="4" t="inlineStr">
+      <c r="G19" s="4" t="inlineStr">
         <is>
           <t>포인트</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="6" t="inlineStr">
-        <is>
-          <t>운행차량 대수</t>
-        </is>
-      </c>
-      <c r="B18" s="6" t="inlineStr">
-        <is>
-          <t>일별 운행 차량 수</t>
-        </is>
-      </c>
-      <c r="C18" s="7" t="inlineStr">
-        <is>
-          <t>1.00</t>
-        </is>
-      </c>
-      <c r="D18" s="7" t="inlineStr">
-        <is>
-          <t>1.00</t>
-        </is>
-      </c>
-      <c r="E18" s="7" t="inlineStr">
-        <is>
-          <t>+0.00</t>
-        </is>
-      </c>
-      <c r="F18" s="7" t="inlineStr">
-        <is>
-          <t>+0.0%</t>
-        </is>
-      </c>
-      <c r="G18" s="6" t="inlineStr">
-        <is>
-          <t>특정일 차량 미운행</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="6" t="inlineStr">
-        <is>
-          <t>운행차량 대수</t>
-        </is>
-      </c>
-      <c r="B19" s="6" t="inlineStr">
-        <is>
-          <t>근무 이행률</t>
-        </is>
-      </c>
-      <c r="C19" s="7" t="inlineStr">
-        <is>
-          <t>1.04</t>
-        </is>
-      </c>
-      <c r="D19" s="7" t="inlineStr">
-        <is>
-          <t>1.03</t>
-        </is>
-      </c>
-      <c r="E19" s="7" t="inlineStr">
-        <is>
-          <t>-0.01</t>
-        </is>
-      </c>
-      <c r="F19" s="7" t="inlineStr">
-        <is>
-          <t>-0.5%</t>
-        </is>
-      </c>
-      <c r="G19" s="6" t="inlineStr">
-        <is>
-          <t>기사 근무 미이행</t>
         </is>
       </c>
     </row>
@@ -2980,150 +3054,150 @@
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
+          <t>일별 운행 차량 수</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>1.00</t>
+        </is>
+      </c>
+      <c r="D20" s="7" t="inlineStr">
+        <is>
+          <t>1.00</t>
+        </is>
+      </c>
+      <c r="E20" s="7" t="inlineStr">
+        <is>
+          <t>+0.00</t>
+        </is>
+      </c>
+      <c r="F20" s="7" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
+      <c r="G20" s="6" t="inlineStr">
+        <is>
+          <t>특정일 차량 미운행</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>운행차량 대수</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>근무 이행률</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>1.04</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="inlineStr">
+        <is>
+          <t>1.03</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="inlineStr">
+        <is>
+          <t>-0.01</t>
+        </is>
+      </c>
+      <c r="F21" s="7" t="inlineStr">
+        <is>
+          <t>-0.5%</t>
+        </is>
+      </c>
+      <c r="G21" s="6" t="inlineStr">
+        <is>
+          <t>기사 근무 미이행</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>운행차량 대수</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
           <t>배차실패 건수(일평균)</t>
         </is>
       </c>
-      <c r="C20" s="7" t="inlineStr">
+      <c r="C22" s="7" t="inlineStr">
         <is>
           <t>2.50</t>
         </is>
       </c>
-      <c r="D20" s="7" t="inlineStr">
+      <c r="D22" s="7" t="inlineStr">
         <is>
           <t>0.00</t>
         </is>
       </c>
-      <c r="E20" s="7" t="inlineStr">
+      <c r="E22" s="7" t="inlineStr">
         <is>
           <t>-2.50</t>
         </is>
       </c>
-      <c r="F20" s="7" t="inlineStr">
+      <c r="F22" s="7" t="inlineStr">
         <is>
           <t>-100.0%</t>
         </is>
       </c>
-      <c r="G20" s="6" t="inlineStr">
+      <c r="G22" s="6" t="inlineStr">
         <is>
           <t>차량 감소에 따른 배차 실패 연쇄</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="10" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="10" t="inlineStr">
         <is>
           <t>▼ 평균 대당 운행시간 (-0.4%)</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="4" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
         <is>
           <t>구분</t>
         </is>
       </c>
-      <c r="B23" s="4" t="inlineStr">
+      <c r="B25" s="4" t="inlineStr">
         <is>
           <t>세부지표</t>
         </is>
       </c>
-      <c r="C23" s="4" t="inlineStr">
+      <c r="C25" s="4" t="inlineStr">
         <is>
           <t>비교기간</t>
         </is>
       </c>
-      <c r="D23" s="4" t="inlineStr">
+      <c r="D25" s="4" t="inlineStr">
         <is>
           <t>분석기간</t>
         </is>
       </c>
-      <c r="E23" s="4" t="inlineStr">
+      <c r="E25" s="4" t="inlineStr">
         <is>
           <t>변동값</t>
         </is>
       </c>
-      <c r="F23" s="4" t="inlineStr">
+      <c r="F25" s="4" t="inlineStr">
         <is>
           <t>변동률</t>
         </is>
       </c>
-      <c r="G23" s="4" t="inlineStr">
+      <c r="G25" s="4" t="inlineStr">
         <is>
           <t>포인트</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="6" t="inlineStr">
-        <is>
-          <t>평균 대당 운행시간</t>
-        </is>
-      </c>
-      <c r="B24" s="6" t="inlineStr">
-        <is>
-          <t>차량별 운행 시간</t>
-        </is>
-      </c>
-      <c r="C24" s="7" t="inlineStr">
-        <is>
-          <t>7.40</t>
-        </is>
-      </c>
-      <c r="D24" s="7" t="inlineStr">
-        <is>
-          <t>7.40</t>
-        </is>
-      </c>
-      <c r="E24" s="7" t="inlineStr">
-        <is>
-          <t>+0.00</t>
-        </is>
-      </c>
-      <c r="F24" s="7" t="inlineStr">
-        <is>
-          <t>+0.0%</t>
-        </is>
-      </c>
-      <c r="G24" s="6" t="inlineStr">
-        <is>
-          <t>특정 차량 운행 시간 편차</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="6" t="inlineStr">
-        <is>
-          <t>평균 대당 운행시간</t>
-        </is>
-      </c>
-      <c r="B25" s="6" t="inlineStr">
-        <is>
-          <t>평균 근무시간</t>
-        </is>
-      </c>
-      <c r="C25" s="7" t="inlineStr">
-        <is>
-          <t>9.36</t>
-        </is>
-      </c>
-      <c r="D25" s="7" t="inlineStr">
-        <is>
-          <t>9.30</t>
-        </is>
-      </c>
-      <c r="E25" s="7" t="inlineStr">
-        <is>
-          <t>-0.05</t>
-        </is>
-      </c>
-      <c r="F25" s="7" t="inlineStr">
-        <is>
-          <t>-0.5%</t>
-        </is>
-      </c>
-      <c r="G25" s="6" t="inlineStr">
-        <is>
-          <t>공차 대기 시간 증가</t>
         </is>
       </c>
     </row>
@@ -3135,150 +3209,150 @@
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
+          <t>차량별 운행 시간</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>7.40</t>
+        </is>
+      </c>
+      <c r="D26" s="7" t="inlineStr">
+        <is>
+          <t>7.40</t>
+        </is>
+      </c>
+      <c r="E26" s="7" t="inlineStr">
+        <is>
+          <t>+0.00</t>
+        </is>
+      </c>
+      <c r="F26" s="7" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
+      <c r="G26" s="6" t="inlineStr">
+        <is>
+          <t>특정 차량 운행 시간 편차</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>평균 대당 운행시간</t>
+        </is>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>평균 근무시간</t>
+        </is>
+      </c>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>9.36</t>
+        </is>
+      </c>
+      <c r="D27" s="7" t="inlineStr">
+        <is>
+          <t>9.30</t>
+        </is>
+      </c>
+      <c r="E27" s="7" t="inlineStr">
+        <is>
+          <t>-0.05</t>
+        </is>
+      </c>
+      <c r="F27" s="7" t="inlineStr">
+        <is>
+          <t>-0.5%</t>
+        </is>
+      </c>
+      <c r="G27" s="6" t="inlineStr">
+        <is>
+          <t>공차 대기 시간 증가</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t>평균 대당 운행시간</t>
+        </is>
+      </c>
+      <c r="B28" s="6" t="inlineStr">
+        <is>
           <t>차량 대당 탑승객</t>
         </is>
       </c>
-      <c r="C26" s="7" t="inlineStr">
+      <c r="C28" s="7" t="inlineStr">
         <is>
           <t>9.50</t>
         </is>
       </c>
-      <c r="D26" s="7" t="inlineStr">
+      <c r="D28" s="7" t="inlineStr">
         <is>
           <t>7.00</t>
         </is>
       </c>
-      <c r="E26" s="7" t="inlineStr">
+      <c r="E28" s="7" t="inlineStr">
         <is>
           <t>-2.50</t>
         </is>
       </c>
-      <c r="F26" s="7" t="inlineStr">
+      <c r="F28" s="7" t="inlineStr">
         <is>
           <t>-26.3%</t>
         </is>
       </c>
-      <c r="G26" s="6" t="inlineStr">
+      <c r="G28" s="6" t="inlineStr">
         <is>
           <t>수요 감소에 따른 공회전</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="10" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="10" t="inlineStr">
         <is>
           <t>▲ 가호출 성공률 (+127.0%)</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="4" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
         <is>
           <t>구분</t>
         </is>
       </c>
-      <c r="B29" s="4" t="inlineStr">
+      <c r="B31" s="4" t="inlineStr">
         <is>
           <t>세부지표</t>
         </is>
       </c>
-      <c r="C29" s="4" t="inlineStr">
+      <c r="C31" s="4" t="inlineStr">
         <is>
           <t>비교기간</t>
         </is>
       </c>
-      <c r="D29" s="4" t="inlineStr">
+      <c r="D31" s="4" t="inlineStr">
         <is>
           <t>분석기간</t>
         </is>
       </c>
-      <c r="E29" s="4" t="inlineStr">
+      <c r="E31" s="4" t="inlineStr">
         <is>
           <t>변동값</t>
         </is>
       </c>
-      <c r="F29" s="4" t="inlineStr">
+      <c r="F31" s="4" t="inlineStr">
         <is>
           <t>변동률</t>
         </is>
       </c>
-      <c r="G29" s="4" t="inlineStr">
+      <c r="G31" s="4" t="inlineStr">
         <is>
           <t>포인트</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="6" t="inlineStr">
-        <is>
-          <t>가호출 성공률</t>
-        </is>
-      </c>
-      <c r="B30" s="6" t="inlineStr">
-        <is>
-          <t>피크 시간대(15~17시) 가호출 성공률</t>
-        </is>
-      </c>
-      <c r="C30" s="7" t="inlineStr">
-        <is>
-          <t>51.4%</t>
-        </is>
-      </c>
-      <c r="D30" s="7" t="inlineStr">
-        <is>
-          <t>77.1%</t>
-        </is>
-      </c>
-      <c r="E30" s="7" t="inlineStr">
-        <is>
-          <t>+25.7%p</t>
-        </is>
-      </c>
-      <c r="F30" s="7" t="inlineStr">
-        <is>
-          <t>+49.9%</t>
-        </is>
-      </c>
-      <c r="G30" s="6" t="inlineStr">
-        <is>
-          <t>피크 시간대 가호출 성공률 변화</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="6" t="inlineStr">
-        <is>
-          <t>가호출 성공률</t>
-        </is>
-      </c>
-      <c r="B31" s="6" t="inlineStr">
-        <is>
-          <t>가호출 성공/실패 회원(일평균)</t>
-        </is>
-      </c>
-      <c r="C31" s="7" t="inlineStr">
-        <is>
-          <t>6.00</t>
-        </is>
-      </c>
-      <c r="D31" s="7" t="inlineStr">
-        <is>
-          <t>3.50</t>
-        </is>
-      </c>
-      <c r="E31" s="7" t="inlineStr">
-        <is>
-          <t>-2.50</t>
-        </is>
-      </c>
-      <c r="F31" s="7" t="inlineStr">
-        <is>
-          <t>-41.7%</t>
-        </is>
-      </c>
-      <c r="G31" s="6" t="inlineStr">
-        <is>
-          <t>가호출 실패 경험 이용자 증가</t>
         </is>
       </c>
     </row>
@@ -3290,32 +3364,32 @@
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>운행차량 대수</t>
+          <t>가호출 성공률(평일)</t>
         </is>
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>1.00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>1.00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E32" s="7" t="inlineStr">
         <is>
-          <t>+0.00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F32" s="7" t="inlineStr">
         <is>
-          <t>+0.0%</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
-          <t>차량 공급 부족에 따른 매칭 실패</t>
+          <t>평일 가호출 성공률 변화</t>
         </is>
       </c>
     </row>
@@ -3327,266 +3401,414 @@
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>가호출 수</t>
+          <t>가호출 성공률(주말)</t>
         </is>
       </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>9.50</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D33" s="7" t="inlineStr">
         <is>
-          <t>7.50</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E33" s="7" t="inlineStr">
         <is>
-          <t>-2.00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F33" s="7" t="inlineStr">
         <is>
-          <t>-21.1%</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G33" s="6" t="inlineStr">
         <is>
-          <t>수요 급증 대비 공급 부족</t>
+          <t>주말 가호출 성공률 변화</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="inlineStr">
+        <is>
+          <t>가호출 성공률</t>
+        </is>
+      </c>
+      <c r="B34" s="6" t="inlineStr">
+        <is>
+          <t>피크 시간대(15~17시) 가호출 성공률</t>
+        </is>
+      </c>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>51.4%</t>
+        </is>
+      </c>
+      <c r="D34" s="7" t="inlineStr">
+        <is>
+          <t>77.1%</t>
+        </is>
+      </c>
+      <c r="E34" s="7" t="inlineStr">
+        <is>
+          <t>+25.7%p</t>
+        </is>
+      </c>
+      <c r="F34" s="7" t="inlineStr">
+        <is>
+          <t>+49.9%</t>
+        </is>
+      </c>
+      <c r="G34" s="6" t="inlineStr">
+        <is>
+          <t>피크 시간대 가호출 성공률 변화</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="10" t="inlineStr">
-        <is>
-          <t>▲ 평균 경로이탈비중 (+3.8%)</t>
+      <c r="A35" s="6" t="inlineStr">
+        <is>
+          <t>가호출 성공률</t>
+        </is>
+      </c>
+      <c r="B35" s="6" t="inlineStr">
+        <is>
+          <t>가호출 성공/실패 회원(일평균)</t>
+        </is>
+      </c>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>6.00</t>
+        </is>
+      </c>
+      <c r="D35" s="7" t="inlineStr">
+        <is>
+          <t>3.50</t>
+        </is>
+      </c>
+      <c r="E35" s="7" t="inlineStr">
+        <is>
+          <t>-2.50</t>
+        </is>
+      </c>
+      <c r="F35" s="7" t="inlineStr">
+        <is>
+          <t>-41.7%</t>
+        </is>
+      </c>
+      <c r="G35" s="6" t="inlineStr">
+        <is>
+          <t>가호출 실패 경험 이용자 증가</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="4" t="inlineStr">
-        <is>
-          <t>구분</t>
-        </is>
-      </c>
-      <c r="B36" s="4" t="inlineStr">
-        <is>
-          <t>세부지표</t>
-        </is>
-      </c>
-      <c r="C36" s="4" t="inlineStr">
-        <is>
-          <t>비교기간</t>
-        </is>
-      </c>
-      <c r="D36" s="4" t="inlineStr">
-        <is>
-          <t>분석기간</t>
-        </is>
-      </c>
-      <c r="E36" s="4" t="inlineStr">
-        <is>
-          <t>변동값</t>
-        </is>
-      </c>
-      <c r="F36" s="4" t="inlineStr">
-        <is>
-          <t>변동률</t>
-        </is>
-      </c>
-      <c r="G36" s="4" t="inlineStr">
-        <is>
-          <t>포인트</t>
+      <c r="A36" s="6" t="inlineStr">
+        <is>
+          <t>가호출 성공률</t>
+        </is>
+      </c>
+      <c r="B36" s="6" t="inlineStr">
+        <is>
+          <t>운행차량 대수</t>
+        </is>
+      </c>
+      <c r="C36" s="7" t="inlineStr">
+        <is>
+          <t>1.00</t>
+        </is>
+      </c>
+      <c r="D36" s="7" t="inlineStr">
+        <is>
+          <t>1.00</t>
+        </is>
+      </c>
+      <c r="E36" s="7" t="inlineStr">
+        <is>
+          <t>+0.00</t>
+        </is>
+      </c>
+      <c r="F36" s="7" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
+      <c r="G36" s="6" t="inlineStr">
+        <is>
+          <t>차량 공급 부족에 따른 매칭 실패</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
+          <t>가호출 성공률</t>
+        </is>
+      </c>
+      <c r="B37" s="6" t="inlineStr">
+        <is>
+          <t>가호출 수(일평균)</t>
+        </is>
+      </c>
+      <c r="C37" s="7" t="inlineStr">
+        <is>
+          <t>9.50</t>
+        </is>
+      </c>
+      <c r="D37" s="7" t="inlineStr">
+        <is>
+          <t>7.50</t>
+        </is>
+      </c>
+      <c r="E37" s="7" t="inlineStr">
+        <is>
+          <t>-2.00</t>
+        </is>
+      </c>
+      <c r="F37" s="7" t="inlineStr">
+        <is>
+          <t>-21.1%</t>
+        </is>
+      </c>
+      <c r="G37" s="6" t="inlineStr">
+        <is>
+          <t>수요 급증 대비 공급 부족</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="10" t="inlineStr">
+        <is>
+          <t>▲ 평균 경로이탈비중 (+3.8%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>구분</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>세부지표</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>비교기간</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>분석기간</t>
+        </is>
+      </c>
+      <c r="E40" s="4" t="inlineStr">
+        <is>
+          <t>변동값</t>
+        </is>
+      </c>
+      <c r="F40" s="4" t="inlineStr">
+        <is>
+          <t>변동률</t>
+        </is>
+      </c>
+      <c r="G40" s="4" t="inlineStr">
+        <is>
+          <t>포인트</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="6" t="inlineStr">
+        <is>
           <t>평균 경로이탈비중</t>
         </is>
       </c>
-      <c r="B37" s="6" t="inlineStr">
+      <c r="B41" s="6" t="inlineStr">
         <is>
           <t>평균 우회비율</t>
         </is>
       </c>
-      <c r="C37" s="7" t="inlineStr">
+      <c r="C41" s="7" t="inlineStr">
         <is>
           <t>0.94</t>
         </is>
       </c>
-      <c r="D37" s="7" t="inlineStr">
+      <c r="D41" s="7" t="inlineStr">
         <is>
           <t>1.07</t>
         </is>
       </c>
-      <c r="E37" s="7" t="inlineStr">
+      <c r="E41" s="7" t="inlineStr">
         <is>
           <t>+0.13</t>
         </is>
       </c>
-      <c r="F37" s="7" t="inlineStr">
+      <c r="F41" s="7" t="inlineStr">
         <is>
           <t>+13.7%</t>
         </is>
       </c>
-      <c r="G37" s="6" t="inlineStr">
+      <c r="G41" s="6" t="inlineStr">
         <is>
           <t>경로 이탈이 우회비율 증가 유발</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="6" t="inlineStr">
-        <is>
-          <t>평균 경로이탈비중</t>
-        </is>
-      </c>
-      <c r="B38" s="6" t="inlineStr">
-        <is>
-          <t>평균 이동시간</t>
-        </is>
-      </c>
-      <c r="C38" s="7" t="inlineStr">
-        <is>
-          <t>10.3</t>
-        </is>
-      </c>
-      <c r="D38" s="7" t="inlineStr">
-        <is>
-          <t>10.4</t>
-        </is>
-      </c>
-      <c r="E38" s="7" t="inlineStr">
-        <is>
-          <t>+0.17</t>
-        </is>
-      </c>
-      <c r="F38" s="7" t="inlineStr">
-        <is>
-          <t>+1.7%</t>
-        </is>
-      </c>
-      <c r="G38" s="6" t="inlineStr">
-        <is>
-          <t>경로 이탈이 이동시간 증가 유발</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="10" t="inlineStr">
-        <is>
-          <t>─ 신규 지역 회원(일평균) (+0.0%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="4" t="inlineStr">
-        <is>
-          <t>구분</t>
-        </is>
-      </c>
-      <c r="B41" s="4" t="inlineStr">
-        <is>
-          <t>세부지표</t>
-        </is>
-      </c>
-      <c r="C41" s="4" t="inlineStr">
-        <is>
-          <t>비교기간</t>
-        </is>
-      </c>
-      <c r="D41" s="4" t="inlineStr">
-        <is>
-          <t>분석기간</t>
-        </is>
-      </c>
-      <c r="E41" s="4" t="inlineStr">
-        <is>
-          <t>변동값</t>
-        </is>
-      </c>
-      <c r="F41" s="4" t="inlineStr">
-        <is>
-          <t>변동률</t>
-        </is>
-      </c>
-      <c r="G41" s="4" t="inlineStr">
-        <is>
-          <t>포인트</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
+          <t>평균 경로이탈비중</t>
+        </is>
+      </c>
+      <c r="B42" s="6" t="inlineStr">
+        <is>
+          <t>평균 이동시간</t>
+        </is>
+      </c>
+      <c r="C42" s="7" t="inlineStr">
+        <is>
+          <t>10.3</t>
+        </is>
+      </c>
+      <c r="D42" s="7" t="inlineStr">
+        <is>
+          <t>10.4</t>
+        </is>
+      </c>
+      <c r="E42" s="7" t="inlineStr">
+        <is>
+          <t>+0.17</t>
+        </is>
+      </c>
+      <c r="F42" s="7" t="inlineStr">
+        <is>
+          <t>+1.7%</t>
+        </is>
+      </c>
+      <c r="G42" s="6" t="inlineStr">
+        <is>
+          <t>경로 이탈이 이동시간 증가 유발</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="10" t="inlineStr">
+        <is>
+          <t>─ 신규 지역 회원(일평균) (+0.0%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>구분</t>
+        </is>
+      </c>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>세부지표</t>
+        </is>
+      </c>
+      <c r="C45" s="4" t="inlineStr">
+        <is>
+          <t>비교기간</t>
+        </is>
+      </c>
+      <c r="D45" s="4" t="inlineStr">
+        <is>
+          <t>분석기간</t>
+        </is>
+      </c>
+      <c r="E45" s="4" t="inlineStr">
+        <is>
+          <t>변동값</t>
+        </is>
+      </c>
+      <c r="F45" s="4" t="inlineStr">
+        <is>
+          <t>변동률</t>
+        </is>
+      </c>
+      <c r="G45" s="4" t="inlineStr">
+        <is>
+          <t>포인트</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="6" t="inlineStr">
+        <is>
           <t>신규 지역 회원(일평균)</t>
         </is>
       </c>
-      <c r="B42" s="6" t="inlineStr">
+      <c r="B46" s="6" t="inlineStr">
         <is>
           <t>누적 지역 회원(일평균)</t>
         </is>
       </c>
-      <c r="C42" s="7" t="inlineStr">
+      <c r="C46" s="7" t="inlineStr">
         <is>
           <t>20.0</t>
         </is>
       </c>
-      <c r="D42" s="7" t="inlineStr">
+      <c r="D46" s="7" t="inlineStr">
         <is>
           <t>25.0</t>
         </is>
       </c>
-      <c r="E42" s="7" t="inlineStr">
+      <c r="E46" s="7" t="inlineStr">
         <is>
           <t>+5.00</t>
         </is>
       </c>
-      <c r="F42" s="7" t="inlineStr">
+      <c r="F46" s="7" t="inlineStr">
         <is>
           <t>+25.0%</t>
         </is>
       </c>
-      <c r="G42" s="6" t="inlineStr">
+      <c r="G46" s="6" t="inlineStr">
         <is>
           <t>전체 회원 기반 성장세</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="6" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="6" t="inlineStr">
         <is>
           <t>신규 지역 회원(일평균)</t>
         </is>
       </c>
-      <c r="B43" s="6" t="inlineStr">
+      <c r="B47" s="6" t="inlineStr">
         <is>
           <t>가호출 순 회원(일평균)</t>
         </is>
       </c>
-      <c r="C43" s="7" t="inlineStr">
+      <c r="C47" s="7" t="inlineStr">
         <is>
           <t>4.00</t>
         </is>
       </c>
-      <c r="D43" s="7" t="inlineStr">
+      <c r="D47" s="7" t="inlineStr">
         <is>
           <t>3.50</t>
         </is>
       </c>
-      <c r="E43" s="7" t="inlineStr">
+      <c r="E47" s="7" t="inlineStr">
         <is>
           <t>-0.50</t>
         </is>
       </c>
-      <c r="F43" s="7" t="inlineStr">
+      <c r="F47" s="7" t="inlineStr">
         <is>
           <t>-12.5%</t>
         </is>
       </c>
-      <c r="G43" s="6" t="inlineStr">
+      <c r="G47" s="6" t="inlineStr">
         <is>
           <t>가입 후 미이용(잠재 이탈) 회원</t>
         </is>
@@ -3594,14 +3816,14 @@
     </row>
   </sheetData>
   <mergeCells count="8">
+    <mergeCell ref="A44:G44"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A40:G40"/>
+    <mergeCell ref="A18:G18"/>
     <mergeCell ref="A3:G3"/>
-    <mergeCell ref="A22:G22"/>
-    <mergeCell ref="A35:G35"/>
-    <mergeCell ref="A16:G16"/>
-    <mergeCell ref="A10:G10"/>
-    <mergeCell ref="A28:G28"/>
+    <mergeCell ref="A39:G39"/>
+    <mergeCell ref="A12:G12"/>
+    <mergeCell ref="A24:G24"/>
+    <mergeCell ref="A30:G30"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>